<commit_message>
[ OK ]  Ahora los archivos de Excel se generan desde variables estaticas la primera vez que se ejecuta Marimo. Se elimina del tracking la carpeta de reporte/
</commit_message>
<xml_diff>
--- a/models/plantilla_informe_he.xlsx
+++ b/models/plantilla_informe_he.xlsx
@@ -817,9 +817,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>109080</xdr:colOff>
+      <xdr:colOff>108720</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>1054080</xdr:rowOff>
+      <xdr:rowOff>1053720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -833,7 +833,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2038320" cy="1054080"/>
+          <a:ext cx="2037960" cy="1053720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -855,9 +855,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>7869960</xdr:colOff>
+      <xdr:colOff>7869600</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>399600</xdr:rowOff>
+      <xdr:rowOff>399240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -871,7 +871,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10010520" y="21960"/>
-          <a:ext cx="4149720" cy="377640"/>
+          <a:ext cx="4149360" cy="377280"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1006,7 +1006,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="6.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="9.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="101.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7.9"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="11" style="1" width="7.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="8.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="3.3"/>

</xml_diff>